<commit_message>
updated calculation for 2D-1C loadcase (which was previously not ideal)
</commit_message>
<xml_diff>
--- a/05_Deploying/error_calc_eps.xlsx
+++ b/05_Deploying/error_calc_eps.xlsx
@@ -714,13 +714,13 @@
         <v>0.145691080489498</v>
       </c>
       <c r="E9" t="n">
-        <v>0.03391172017343642</v>
+        <v>0.02075120592637849</v>
       </c>
       <c r="F9" t="n">
-        <v>15.80776553539411</v>
+        <v>0.1029938431312478</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0594147606759236</v>
+        <v>0.07525593479458105</v>
       </c>
       <c r="H9" t="n">
         <v>0.004003558522657017</v>

</xml_diff>

<commit_message>
added getting maximum values for every strain and displ path for table in appendix
</commit_message>
<xml_diff>
--- a/05_Deploying/error_calc_eps.xlsx
+++ b/05_Deploying/error_calc_eps.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -565,409 +565,851 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>2D-2</t>
+          <t>2D-1</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0006536362429842648</v>
+        <v>4.141608907906138</v>
       </c>
       <c r="C5" t="n">
-        <v>0.07914788431458994</v>
+        <v>4.14160890789241</v>
       </c>
       <c r="D5" t="n">
-        <v>0.03615232067351627</v>
+        <v>8.999277915709795</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0006442912702896891</v>
+        <v>2.370985131798637</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1651239159894753</v>
+        <v>3.400920733699106</v>
       </c>
       <c r="G5" t="n">
-        <v>0.04232368565908246</v>
+        <v>6.237132720724544</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0004720678215408128</v>
+        <v>5.926335134026517</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1816128675968975</v>
+        <v>3.829969163366695</v>
       </c>
       <c r="J5" t="n">
-        <v>0.04323971224691036</v>
+        <v>10.5472003018754</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>2D-3</t>
+          <t>2D-2</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.000437873356409088</v>
+        <v>0.0006536362429842648</v>
       </c>
       <c r="C6" t="n">
-        <v>0.02962605541802788</v>
+        <v>0.07914788431458994</v>
       </c>
       <c r="D6" t="n">
-        <v>0.003734938431332921</v>
+        <v>0.03615232067351627</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0003016260968178915</v>
+        <v>0.0006442912702896891</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0116702176835575</v>
+        <v>0.1651239159894753</v>
       </c>
       <c r="G6" t="n">
-        <v>0.002350717616909167</v>
+        <v>0.04232368565908246</v>
       </c>
       <c r="H6" t="n">
-        <v>0.0001484086212952306</v>
+        <v>0.0004720678215408128</v>
       </c>
       <c r="I6" t="n">
-        <v>0.01582774170278483</v>
+        <v>0.1816128675968975</v>
       </c>
       <c r="J6" t="n">
-        <v>0.003698944645119666</v>
+        <v>0.04323971224691036</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>2D-4</t>
+          <t>2D-2</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.1615566082410709</v>
+        <v>0.00280895868685783</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0007502766592417921</v>
+        <v>4.141608908008186</v>
       </c>
       <c r="D7" t="n">
-        <v>0.03423619286373029</v>
+        <v>3.095931222838041e-10</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1737041834172787</v>
+        <v>0.002808684633796813</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0002971605144958956</v>
+        <v>3.31939064922318</v>
       </c>
       <c r="G7" t="n">
-        <v>0.02633395640970925</v>
+        <v>1.852538508337852e-10</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1023184120166581</v>
+        <v>0.002808802755565744</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0004440832050434508</v>
+        <v>3.688503302949742</v>
       </c>
       <c r="J7" t="n">
-        <v>0.02507745363225094</v>
+        <v>4.830354027529561e-10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>2D-5</t>
+          <t>2D-3</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.04071387600736533</v>
+        <v>0.000437873356409088</v>
       </c>
       <c r="C8" t="n">
-        <v>0.000617185595694431</v>
+        <v>0.02962605541802788</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0008163681706247216</v>
+        <v>0.003734938431332921</v>
       </c>
       <c r="E8" t="n">
-        <v>0.03390245384500636</v>
+        <v>0.0003016260968178915</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0006062956834057625</v>
+        <v>0.0116702176835575</v>
       </c>
       <c r="G8" t="n">
-        <v>0.000666410056720204</v>
+        <v>0.002350717616909167</v>
       </c>
       <c r="H8" t="n">
-        <v>0.03389399066638887</v>
+        <v>0.0001484086212952306</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0006290298886622074</v>
+        <v>0.01582774170278483</v>
       </c>
       <c r="J8" t="n">
-        <v>0.0005156025109879299</v>
+        <v>0.003698944645119666</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>2D-1C</t>
+          <t>2D-3</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.2019197655991049</v>
+        <v>0.002834909414587643</v>
       </c>
       <c r="C9" t="n">
-        <v>0.1847320988047952</v>
+        <v>2.177577525062954</v>
       </c>
       <c r="D9" t="n">
-        <v>0.145691080489498</v>
+        <v>4.764230904241118e-07</v>
       </c>
       <c r="E9" t="n">
-        <v>0.02075120592637849</v>
+        <v>0.002834909414440349</v>
       </c>
       <c r="F9" t="n">
-        <v>0.1029938431312478</v>
+        <v>1.574322617235925</v>
       </c>
       <c r="G9" t="n">
-        <v>0.07525593479458105</v>
+        <v>2.300026169252273e-07</v>
       </c>
       <c r="H9" t="n">
-        <v>0.004003558522657017</v>
+        <v>0.002834909414459152</v>
       </c>
       <c r="I9" t="n">
-        <v>0.0209457929564454</v>
+        <v>1.809308418047418</v>
       </c>
       <c r="J9" t="n">
-        <v>0.05077887174956273</v>
+        <v>4.766630315578867e-07</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>2D-2C</t>
+          <t>2D-4</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.2433902032696133</v>
+        <v>0.1615566082410709</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0009224800648023682</v>
+        <v>0.0007502766592417921</v>
       </c>
       <c r="D10" t="n">
-        <v>0.009894444946539393</v>
+        <v>0.03423619286373029</v>
       </c>
       <c r="E10" t="n">
-        <v>0.166733947367969</v>
+        <v>0.1737041834172787</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0006632263887096515</v>
+        <v>0.0002971605144958956</v>
       </c>
       <c r="G10" t="n">
-        <v>0.01520362369963257</v>
+        <v>0.02633395640970925</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1354023846642725</v>
+        <v>0.1023184120166581</v>
       </c>
       <c r="I10" t="n">
-        <v>0.0008488519998968035</v>
+        <v>0.0004440832050434508</v>
       </c>
       <c r="J10" t="n">
-        <v>0.008588589444195499</v>
+        <v>0.02507745363225094</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>2D-3C</t>
+          <t>2D-4</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.2969467336996298</v>
+        <v>4.14160890815693</v>
       </c>
       <c r="C11" t="n">
-        <v>0.7160121635999773</v>
+        <v>0.002808958687000284</v>
       </c>
       <c r="D11" t="n">
-        <v>0.9299834464147567</v>
+        <v>4.444768897996474e-09</v>
       </c>
       <c r="E11" t="n">
-        <v>0.1507189158917917</v>
+        <v>4.141608908104761</v>
       </c>
       <c r="F11" t="n">
-        <v>0.7141942297687615</v>
+        <v>0.002850045750058933</v>
       </c>
       <c r="G11" t="n">
-        <v>0.6611442967201387</v>
+        <v>4.474217469704e-09</v>
       </c>
       <c r="H11" t="n">
-        <v>0.03768493609280239</v>
+        <v>4.14160890826332</v>
       </c>
       <c r="I11" t="n">
-        <v>0.04396534397697937</v>
+        <v>0.002730243446063024</v>
       </c>
       <c r="J11" t="n">
-        <v>0.08026617014866609</v>
+        <v>4.38830500834131e-09</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>2D-4C</t>
+          <t>2D-5</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.01122561227979022</v>
+        <v>0.04071387600736533</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0074539018580184</v>
+        <v>0.000617185595694431</v>
       </c>
       <c r="D12" t="n">
-        <v>0.02681945586741276</v>
+        <v>0.0008163681706247216</v>
       </c>
       <c r="E12" t="n">
-        <v>0.01507311002828347</v>
+        <v>0.03390245384500636</v>
       </c>
       <c r="F12" t="n">
-        <v>2.514915027865713</v>
+        <v>0.0006062956834057625</v>
       </c>
       <c r="G12" t="n">
-        <v>0.008031236504127653</v>
+        <v>0.000666410056720204</v>
       </c>
       <c r="H12" t="n">
-        <v>0.5007775954964752</v>
+        <v>0.03389399066638887</v>
       </c>
       <c r="I12" t="n">
-        <v>0.003687851307946168</v>
+        <v>0.0006290298886622074</v>
       </c>
       <c r="J12" t="n">
-        <v>0.003673202081335721</v>
+        <v>0.0005156025109879299</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>2D-5C</t>
+          <t>2D-5</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1101524278711081</v>
+        <v>2.177577525058719</v>
       </c>
       <c r="C13" t="n">
-        <v>0.03080486046493565</v>
+        <v>0.002834909414443699</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1221199231668258</v>
+        <v>1.369354628332538e-11</v>
       </c>
       <c r="E13" t="n">
-        <v>1.110492666840618</v>
+        <v>2.177577525058803</v>
       </c>
       <c r="F13" t="n">
-        <v>0.8711624815926103</v>
+        <v>0.002876753020873879</v>
       </c>
       <c r="G13" t="n">
-        <v>3.719303625982536</v>
+        <v>1.366851222456928e-11</v>
       </c>
       <c r="H13" t="n">
-        <v>0.05826785587015933</v>
+        <v>2.177577525058563</v>
       </c>
       <c r="I13" t="n">
-        <v>0.02093932903835912</v>
+        <v>0.002754774521147356</v>
       </c>
       <c r="J13" t="n">
-        <v>0.07543583057939422</v>
+        <v>1.374053797717316e-11</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>2D-6C</t>
+          <t>2D-1C</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.03737690827971605</v>
+        <v>0.2019197655991049</v>
       </c>
       <c r="C14" t="n">
-        <v>0.02761967379203449</v>
+        <v>0.1847320988047952</v>
       </c>
       <c r="D14" t="n">
-        <v>0.06390377387519114</v>
+        <v>0.145691080489498</v>
       </c>
       <c r="E14" t="n">
-        <v>0.03101240078147507</v>
+        <v>0.02075120592637849</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0395390521089547</v>
+        <v>0.1029938431312478</v>
       </c>
       <c r="G14" t="n">
-        <v>0.06463821255783096</v>
+        <v>0.07525593479458105</v>
       </c>
       <c r="H14" t="n">
-        <v>0.072222749579112</v>
+        <v>0.004003558522657017</v>
       </c>
       <c r="I14" t="n">
-        <v>0.03373121744450615</v>
+        <v>0.0209457929564454</v>
       </c>
       <c r="J14" t="n">
-        <v>0.09837024195774073</v>
+        <v>0.05077887174956273</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>2D-7C</t>
+          <t>2D-1C</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.008395621979728355</v>
+        <v>4.141127676376564</v>
       </c>
       <c r="C15" t="n">
-        <v>0.009644239468249679</v>
+        <v>4.141127676261973</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0266117600914953</v>
+        <v>1.370193888905469e-09</v>
       </c>
       <c r="E15" t="n">
-        <v>0.01907736154419423</v>
+        <v>1.522487695187477</v>
       </c>
       <c r="F15" t="n">
-        <v>0.01991550694012741</v>
+        <v>3.319029846910527</v>
       </c>
       <c r="G15" t="n">
-        <v>0.04222562226803962</v>
+        <v>7.513291204463979e-10</v>
       </c>
       <c r="H15" t="n">
-        <v>0.009327616477616254</v>
+        <v>1.766388944447298</v>
       </c>
       <c r="I15" t="n">
-        <v>0.009001022393814654</v>
+        <v>1.179174214068691</v>
       </c>
       <c r="J15" t="n">
-        <v>0.02118758831484774</v>
+        <v>4.845559717359116e-10</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
+          <t>2D-2C</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.2433902032696133</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.0009224800648023682</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.009894444946539393</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.166733947367969</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.0006632263887096515</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.01520362369963257</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.1354023846642725</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.0008488519998968035</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.008588589444195499</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>2D-2C</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>4.141608908154494</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.1413206045445593</v>
+      </c>
+      <c r="D17" t="n">
+        <v>8.275898079356837e-08</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3.77112645598507</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.1422512824131193</v>
+      </c>
+      <c r="G17" t="n">
+        <v>7.557566006929743e-08</v>
+      </c>
+      <c r="H17" t="n">
+        <v>4.141608908260876</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.1368027364421629</v>
+      </c>
+      <c r="J17" t="n">
+        <v>8.045621054152477e-08</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>2D-3C</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.2969467336996298</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.7160121635999773</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.9299834464147567</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.1507189158917917</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.7141942297687615</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.6611442967201387</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.03768493609280239</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.04396534397697937</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.08026617014866609</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>2D-3C</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3.161162505653022</v>
+      </c>
+      <c r="C19" t="n">
+        <v>8.488485259518979</v>
+      </c>
+      <c r="D19" t="n">
+        <v>10.87283798623087</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2.238479343994432</v>
+      </c>
+      <c r="F19" t="n">
+        <v>9.039667061445718</v>
+      </c>
+      <c r="G19" t="n">
+        <v>9.489950840824669</v>
+      </c>
+      <c r="H19" t="n">
+        <v>3.183549270606864</v>
+      </c>
+      <c r="I19" t="n">
+        <v>4.679605284254493</v>
+      </c>
+      <c r="J19" t="n">
+        <v>8.290475467534133</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>2D-4C</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.01122561227979022</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.0074539018580184</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.02681945586741276</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.01507311002828347</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2.514915027865713</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.008031236504127653</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.5007775954964752</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.003687851307946168</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.003673202081335721</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>2D-4C</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2.177577523259924</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2.177577531120621</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1.010136722531807e-08</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1.970924622636809</v>
+      </c>
+      <c r="F21" t="n">
+        <v>8.302407737756473</v>
+      </c>
+      <c r="G21" t="n">
+        <v>8.084414964727726e-07</v>
+      </c>
+      <c r="H21" t="n">
+        <v>3.580268709569723</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1.785945103038507</v>
+      </c>
+      <c r="J21" t="n">
+        <v>1.693901095778383e-10</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>2D-5C</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0.1101524278711081</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.03080486046493565</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.1221199231668258</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1.110492666840618</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.8711624815926103</v>
+      </c>
+      <c r="G22" t="n">
+        <v>3.719303625982536</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.05826785587015933</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.02093932903835912</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.07543583057939422</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>2D-5C</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>5.458682457843471</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1.750095411982064</v>
+      </c>
+      <c r="D23" t="n">
+        <v>8.090107749785691</v>
+      </c>
+      <c r="E23" t="n">
+        <v>6.399839449226532</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2.46604525905338</v>
+      </c>
+      <c r="G23" t="n">
+        <v>9.653558369588515</v>
+      </c>
+      <c r="H23" t="n">
+        <v>4.101025966779638</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1.172985468916958</v>
+      </c>
+      <c r="J23" t="n">
+        <v>6.190210230095037</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>2D-6C</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0.03737690827971605</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.02761967379203449</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.06390377387519114</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.03101240078147507</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.0395390521089547</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.06463821255783096</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.072222749579112</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.03373121744450615</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.09837024195774073</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>2D-6C</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2.425657373814495</v>
+      </c>
+      <c r="C25" t="n">
+        <v>2.425657373812651</v>
+      </c>
+      <c r="D25" t="n">
+        <v>5.251458869002635</v>
+      </c>
+      <c r="E25" t="n">
+        <v>2.684101054201339</v>
+      </c>
+      <c r="F25" t="n">
+        <v>4.04946727737771</v>
+      </c>
+      <c r="G25" t="n">
+        <v>6.96557890032182</v>
+      </c>
+      <c r="H25" t="n">
+        <v>3.853039951360042</v>
+      </c>
+      <c r="I25" t="n">
+        <v>2.124434805826668</v>
+      </c>
+      <c r="J25" t="n">
+        <v>6.281334660472252</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>2D-7C</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0.008395621979728355</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.009644239468249679</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.0266117600914953</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.01907736154419423</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.01991550694012741</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.04222562226803962</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.009327616477616254</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.009001022393814654</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.02118758831484774</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>2D-7C</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.1848219512387388</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.1848219512405593</v>
+      </c>
+      <c r="D27" t="n">
+        <v>2.940836949554776</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.2118032579883685</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.2118032579912279</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2.886873955153844</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.146714332427033</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.1467143324270209</v>
+      </c>
+      <c r="J27" t="n">
+        <v>3.023249552815799</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
           <t>2D-8C</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B28" t="n">
         <v>0.7759858700802337</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C28" t="n">
         <v>0.08511866148315227</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D28" t="n">
         <v>0.5493262796095778</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E28" t="n">
         <v>0.5108114560408168</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F28" t="n">
         <v>0.08445939045119669</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G28" t="n">
         <v>0.4317206469700591</v>
       </c>
-      <c r="H16" t="n">
+      <c r="H28" t="n">
         <v>2.569047687085132</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I28" t="n">
         <v>0.1279102508455969</v>
       </c>
-      <c r="J16" t="n">
+      <c r="J28" t="n">
         <v>1.458503888976329</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>2D-8C</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>9.94365899339563</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1.666402663642911</v>
+      </c>
+      <c r="D29" t="n">
+        <v>9.088154605628207</v>
+      </c>
+      <c r="E29" t="n">
+        <v>9.165282251132147</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1.945813931592985</v>
+      </c>
+      <c r="G29" t="n">
+        <v>9.221200120639095</v>
+      </c>
+      <c r="H29" t="n">
+        <v>18.74872373786611</v>
+      </c>
+      <c r="I29" t="n">
+        <v>1.752070045195834</v>
+      </c>
+      <c r="J29" t="n">
+        <v>13.47025022750447</v>
       </c>
     </row>
   </sheetData>

</xml_diff>